<commit_message>
Adiciona projeto dbt completo, escrow, orquestração e correções de estrutura de pastas
</commit_message>
<xml_diff>
--- a/extraction/planilhas/custo_produtos.xlsx
+++ b/extraction/planilhas/custo_produtos.xlsx
@@ -1,27 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brunoalencar/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brunoalencar/Documents/Casa e Patas/data-pipeline/extraction/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A0E95CF-299F-7C43-B773-0D29097255CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{778EAB7B-9770-AF48-A095-D20D7DF0E9C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30500" yWindow="1360" windowWidth="31060" windowHeight="26840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="custo_produtos" sheetId="1" r:id="rId1"/>
     <sheet name="legenda" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="215">
   <si>
     <t>Custo de Produtos — Casa e Patas</t>
   </si>
@@ -594,6 +607,78 @@
   </si>
   <si>
     <t>Kit 3 Capas Cilindro + Painel Redondo Feliz Aniversário Tecido Premium Floral Rosé</t>
+  </si>
+  <si>
+    <t>TESTE-CASA-PATAS-001</t>
+  </si>
+  <si>
+    <t>Coleira Teste Casa e Patas</t>
+  </si>
+  <si>
+    <t>Custo de Teste</t>
+  </si>
+  <si>
+    <t>46.55</t>
+  </si>
+  <si>
+    <t>52.86</t>
+  </si>
+  <si>
+    <t>65.46</t>
+  </si>
+  <si>
+    <t>33.95</t>
+  </si>
+  <si>
+    <t>24.48</t>
+  </si>
+  <si>
+    <t>12.9</t>
+  </si>
+  <si>
+    <t>10.21</t>
+  </si>
+  <si>
+    <t>7.7</t>
+  </si>
+  <si>
+    <t>7.18</t>
+  </si>
+  <si>
+    <t>13.51</t>
+  </si>
+  <si>
+    <t>52.23</t>
+  </si>
+  <si>
+    <t>5.19</t>
+  </si>
+  <si>
+    <t>20.46</t>
+  </si>
+  <si>
+    <t>16.44</t>
+  </si>
+  <si>
+    <t>29.23</t>
+  </si>
+  <si>
+    <t>6.91</t>
+  </si>
+  <si>
+    <t>9.98</t>
+  </si>
+  <si>
+    <t>68.35</t>
+  </si>
+  <si>
+    <t>8.3</t>
+  </si>
+  <si>
+    <t>44.9</t>
+  </si>
+  <si>
+    <t>24.27</t>
   </si>
 </sst>
 </file>
@@ -616,44 +701,52 @@
       <sz val="14"/>
       <color rgb="FF1F4E78"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF808080"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -711,7 +804,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -720,7 +813,6 @@
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -733,6 +825,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -741,9 +836,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1045,9 +1137,48 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{8FBDB2D1-12AB-BF44-9728-3A4D166D51D3}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;632c5ad1-1611-4f78-9524-212dd47a6297&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{2E2A0FD1-1816-D04B-8B7B-EACF212C71F8}">
+  <we:reference id="WA200010725" version="1.0.0.1" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200010725" version="1.0.0.1" store="WA200010725" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;5ee2d0e2-1201-4b6e-84ee-87f2a87927ff&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J90"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1060,22 +1191,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
     </row>
     <row r="2" spans="1:10" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
@@ -1095,16 +1226,16 @@
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="13">
         <v>33.770000000000003</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="14">
         <v>46174</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -1121,978 +1252,1230 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="13">
         <v>46.3</v>
       </c>
-      <c r="D6" s="6"/>
+      <c r="D6" s="14">
+        <v>46174</v>
+      </c>
       <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="13">
         <v>52.57</v>
       </c>
-      <c r="D7" s="6"/>
+      <c r="D7" s="14">
+        <v>46174</v>
+      </c>
       <c r="E7" s="5"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="13">
         <v>65.099999999999994</v>
       </c>
-      <c r="D8" s="6"/>
+      <c r="D8" s="14">
+        <v>46174</v>
+      </c>
       <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="13">
         <v>33.950000000000003</v>
       </c>
-      <c r="D9" s="6"/>
+      <c r="D9" s="14">
+        <v>46174</v>
+      </c>
       <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="13">
         <v>46.55</v>
       </c>
-      <c r="D10" s="6"/>
+      <c r="D10" s="14">
+        <v>46174</v>
+      </c>
       <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="13">
         <v>52.86</v>
       </c>
-      <c r="D11" s="6"/>
+      <c r="D11" s="14">
+        <v>46174</v>
+      </c>
       <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="13">
         <v>65.459999999999994</v>
       </c>
-      <c r="D12" s="6"/>
+      <c r="D12" s="14">
+        <v>46174</v>
+      </c>
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="13">
         <v>33.950000000000003</v>
       </c>
-      <c r="D13" s="6"/>
+      <c r="D13" s="14">
+        <v>46174</v>
+      </c>
       <c r="E13" s="5"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="C14" s="18">
+      <c r="C14" s="13">
         <v>46.55</v>
       </c>
-      <c r="D14" s="6"/>
+      <c r="D14" s="14">
+        <v>46174</v>
+      </c>
       <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="13">
         <v>52.86</v>
       </c>
-      <c r="D15" s="6"/>
+      <c r="D15" s="14">
+        <v>46174</v>
+      </c>
       <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="13">
         <v>65.459999999999994</v>
       </c>
-      <c r="D16" s="6"/>
+      <c r="D16" s="14">
+        <v>46174</v>
+      </c>
       <c r="E16" s="5"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="13">
         <v>33.950000000000003</v>
       </c>
-      <c r="D17" s="6"/>
+      <c r="D17" s="14">
+        <v>46174</v>
+      </c>
       <c r="E17" s="5"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="13">
         <v>46.55</v>
       </c>
-      <c r="D18" s="6"/>
+      <c r="D18" s="14">
+        <v>46174</v>
+      </c>
       <c r="E18" s="5"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="13">
         <v>52.86</v>
       </c>
-      <c r="D19" s="6"/>
+      <c r="D19" s="14">
+        <v>46174</v>
+      </c>
       <c r="E19" s="5"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="13">
         <v>65.459999999999994</v>
       </c>
-      <c r="D20" s="6"/>
+      <c r="D20" s="14">
+        <v>46174</v>
+      </c>
       <c r="E20" s="5"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="C21" s="18">
+      <c r="C21" s="13">
         <v>33.950000000000003</v>
       </c>
-      <c r="D21" s="6"/>
+      <c r="D21" s="14">
+        <v>46174</v>
+      </c>
       <c r="E21" s="5"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="C22" s="18">
+      <c r="C22" s="13">
         <v>46.55</v>
       </c>
-      <c r="D22" s="6"/>
+      <c r="D22" s="14">
+        <v>46174</v>
+      </c>
       <c r="E22" s="5"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="C23" s="18">
+      <c r="C23" s="13">
         <v>52.86</v>
       </c>
-      <c r="D23" s="6"/>
+      <c r="D23" s="14">
+        <v>46174</v>
+      </c>
       <c r="E23" s="5"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="C24" s="18">
+      <c r="C24" s="13">
         <v>65.459999999999994</v>
       </c>
-      <c r="D24" s="6"/>
+      <c r="D24" s="14">
+        <v>46174</v>
+      </c>
       <c r="E24" s="5"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="C25" s="18">
+      <c r="C25" s="13">
         <v>33.950000000000003</v>
       </c>
-      <c r="D25" s="6"/>
+      <c r="D25" s="14">
+        <v>46174</v>
+      </c>
       <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="C26" s="18">
-        <v>46.55</v>
+      <c r="C26" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D26" s="14">
+        <v>46174</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="C27" s="18">
-        <v>52.86</v>
+      <c r="C27" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D27" s="14">
+        <v>46174</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="17" t="s">
+      <c r="B28" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="C28" s="18">
-        <v>65.459999999999994</v>
+      <c r="C28" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D28" s="14">
+        <v>46174</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="C29" s="18">
-        <v>33.950000000000003</v>
+      <c r="C29" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D29" s="14">
+        <v>46174</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="C30" s="18">
-        <v>46.55</v>
+      <c r="C30" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D30" s="14">
+        <v>46174</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="C31" s="18">
-        <v>52.86</v>
+      <c r="C31" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D31" s="14">
+        <v>46174</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="17" t="s">
+      <c r="A32" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="B32" s="17" t="s">
+      <c r="B32" s="12" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="18">
-        <v>65.459999999999994</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="17" t="s">
+      <c r="C32" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D32" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="C33" s="18">
-        <v>33.950000000000003</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="17" t="s">
+      <c r="C33" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D33" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B34" s="17" t="s">
+      <c r="B34" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="C34" s="18">
-        <v>46.55</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="17" t="s">
+      <c r="C34" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D34" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B35" s="17" t="s">
+      <c r="B35" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="C35" s="18">
-        <v>52.86</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="17" t="s">
+      <c r="C35" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D35" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="17" t="s">
+      <c r="B36" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="C36" s="18">
-        <v>65.459999999999994</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="17" t="s">
+      <c r="C36" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D36" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="C37" s="18">
-        <v>33.950000000000003</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="17" t="s">
+      <c r="C37" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D37" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B38" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="C38" s="18">
-        <v>46.55</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="17" t="s">
+      <c r="C38" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D38" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B39" s="17" t="s">
+      <c r="B39" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="C39" s="18">
-        <v>52.86</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="17" t="s">
+      <c r="C39" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D39" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="C40" s="18">
-        <v>65.459999999999994</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="17" t="s">
+      <c r="C40" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D40" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="C41" s="18">
-        <v>33.950000000000003</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A42" s="17" t="s">
+      <c r="C41" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D41" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="B42" s="17" t="s">
+      <c r="B42" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="C42" s="18">
-        <v>46.55</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A43" s="17" t="s">
+      <c r="C42" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D42" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B43" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="C43" s="18">
-        <v>52.86</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A44" s="17" t="s">
+      <c r="C43" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D43" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B44" s="17" t="s">
+      <c r="B44" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="C44" s="18">
-        <v>65.459999999999994</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A45" s="17" t="s">
+      <c r="C44" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D44" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B45" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="C45" s="18">
-        <v>33.950000000000003</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A46" s="17" t="s">
+      <c r="C45" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D45" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="B46" s="17" t="s">
+      <c r="B46" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="C46" s="18">
-        <v>46.55</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A47" s="17" t="s">
+      <c r="C46" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D46" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="C47" s="18">
-        <v>52.86</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A48" s="17" t="s">
+      <c r="C47" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D47" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="B48" s="17" t="s">
+      <c r="B48" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="C48" s="18">
-        <v>65.459999999999994</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A49" s="17" t="s">
+      <c r="C48" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D48" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="C49" s="18">
-        <v>33.950000000000003</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A50" s="17" t="s">
+      <c r="C49" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D49" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="B50" s="17" t="s">
+      <c r="B50" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="C50" s="18">
-        <v>46.55</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A51" s="17" t="s">
+      <c r="C50" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D50" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B51" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="C51" s="18">
-        <v>52.86</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A52" s="17" t="s">
+      <c r="C51" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D51" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B52" s="17" t="s">
+      <c r="B52" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="C52" s="18">
-        <v>65.459999999999994</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A53" s="17" t="s">
+      <c r="C52" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D52" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B53" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="C53" s="18">
-        <v>24.48</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A54" s="17" t="s">
+      <c r="C53" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="D53" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B54" s="17" t="s">
+      <c r="B54" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="C54" s="18">
-        <v>12.9</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A55" s="17" t="s">
+      <c r="C54" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D54" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="12" t="s">
         <v>69</v>
       </c>
-      <c r="B55" s="17" t="s">
+      <c r="B55" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="C55" s="18">
-        <v>10.210000000000001</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A56" s="17" t="s">
+      <c r="C55" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D55" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="B56" s="17" t="s">
+      <c r="B56" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="C56" s="18">
-        <v>10.210000000000001</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A57" s="17" t="s">
+      <c r="C56" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D56" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B57" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="C57" s="18">
-        <v>10.210000000000001</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="17" t="s">
+      <c r="C57" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D57" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B58" s="17" t="s">
+      <c r="B58" s="12" t="s">
         <v>158</v>
       </c>
-      <c r="C58" s="18">
-        <v>10.210000000000001</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A59" s="17" t="s">
+      <c r="C58" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D58" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B59" s="17" t="s">
+      <c r="B59" s="12" t="s">
         <v>159</v>
       </c>
-      <c r="C59" s="18">
-        <v>7.7</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A60" s="17" t="s">
+      <c r="C59" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="D59" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="B60" s="17" t="s">
+      <c r="B60" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="C60" s="18">
-        <v>7.18</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A61" s="17" t="s">
+      <c r="C60" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D60" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B61" s="17" t="s">
+      <c r="B61" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="C61" s="18">
-        <v>13.51</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A62" s="17" t="s">
+      <c r="C61" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="D61" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="B62" s="17" t="s">
+      <c r="B62" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="C62" s="18">
-        <v>52.23</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A63" s="17" t="s">
+      <c r="C62" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="D62" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="B63" s="17" t="s">
+      <c r="B63" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="C63" s="18">
-        <v>5.19</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A64" s="17" t="s">
+      <c r="C63" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D63" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B64" s="17" t="s">
+      <c r="B64" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="C64" s="18">
-        <v>20.46</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A65" s="17" t="s">
+      <c r="C64" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="D64" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B65" s="17" t="s">
+      <c r="B65" s="12" t="s">
         <v>165</v>
       </c>
-      <c r="C65" s="18">
-        <v>16.440000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A66" s="17" t="s">
+      <c r="C65" s="13" t="s">
+        <v>207</v>
+      </c>
+      <c r="D65" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="B66" s="17" t="s">
+      <c r="B66" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="C66" s="18">
-        <v>29.23</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A67" s="17" t="s">
+      <c r="C66" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="D66" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B67" s="17" t="s">
+      <c r="B67" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="C67" s="18">
-        <v>6.91</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A68" s="17" t="s">
+      <c r="C67" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="D67" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B68" s="17" t="s">
+      <c r="B68" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="C68" s="18">
-        <v>9.98</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A69" s="17" t="s">
+      <c r="C68" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="D68" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B69" s="17" t="s">
+      <c r="B69" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="C69" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A70" s="17" t="s">
+      <c r="C69" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D69" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="B70" s="17" t="s">
+      <c r="B70" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="C70" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A71" s="17" t="s">
+      <c r="C70" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D70" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B71" s="17" t="s">
+      <c r="B71" s="12" t="s">
         <v>171</v>
       </c>
-      <c r="C71" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A72" s="17" t="s">
+      <c r="C71" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D71" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="B72" s="17" t="s">
+      <c r="B72" s="12" t="s">
         <v>172</v>
       </c>
-      <c r="C72" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A73" s="17" t="s">
+      <c r="C72" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D72" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="B73" s="17" t="s">
+      <c r="B73" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="C73" s="18">
-        <v>8.3000000000000007</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A74" s="17" t="s">
+      <c r="C73" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D73" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B74" s="17" t="s">
+      <c r="B74" s="12" t="s">
         <v>174</v>
       </c>
-      <c r="C74" s="18">
-        <v>8.3000000000000007</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A75" s="17" t="s">
+      <c r="C74" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D74" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="B75" s="17" t="s">
+      <c r="B75" s="12" t="s">
         <v>175</v>
       </c>
-      <c r="C75" s="18">
-        <v>8.3000000000000007</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A76" s="17" t="s">
+      <c r="C75" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D75" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B76" s="17" t="s">
+      <c r="B76" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="C76" s="18">
-        <v>8.3000000000000007</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A77" s="17" t="s">
+      <c r="C76" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="D76" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B77" s="17" t="s">
+      <c r="B77" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="C77" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A78" s="17" t="s">
+      <c r="C77" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D77" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="B78" s="17" t="s">
+      <c r="B78" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="C78" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A79" s="17" t="s">
+      <c r="C78" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D78" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="B79" s="17" t="s">
+      <c r="B79" s="12" t="s">
         <v>179</v>
       </c>
-      <c r="C79" s="18">
-        <v>44.9</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A80" s="17" t="s">
+      <c r="C79" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="D79" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="B80" s="17" t="s">
+      <c r="B80" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="C80" s="18">
-        <v>44.9</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A81" s="17" t="s">
+      <c r="C80" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="D80" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A81" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="B81" s="17" t="s">
+      <c r="B81" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="C81" s="18">
-        <v>44.9</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A82" s="17" t="s">
+      <c r="C81" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="D81" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A82" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="B82" s="17" t="s">
+      <c r="B82" s="12" t="s">
         <v>182</v>
       </c>
-      <c r="C82" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A83" s="17" t="s">
+      <c r="C82" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D82" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A83" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="B83" s="17" t="s">
+      <c r="B83" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="C83" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A84" s="17" t="s">
+      <c r="C83" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D83" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A84" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="B84" s="17" t="s">
+      <c r="B84" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="C84" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A85" s="17" t="s">
+      <c r="C84" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D84" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A85" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="B85" s="17" t="s">
+      <c r="B85" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="C85" s="18">
-        <v>24.27</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A86" s="17" t="s">
+      <c r="C85" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D85" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A86" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="B86" s="17" t="s">
+      <c r="B86" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="C86" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A87" s="17" t="s">
+      <c r="C86" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D86" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A87" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="B87" s="17" t="s">
+      <c r="B87" s="12" t="s">
         <v>187</v>
       </c>
-      <c r="C87" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A88" s="17" t="s">
+      <c r="C87" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D87" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A88" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="B88" s="17" t="s">
+      <c r="B88" s="12" t="s">
         <v>188</v>
       </c>
-      <c r="C88" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A89" s="17" t="s">
+      <c r="C88" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D88" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A89" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="B89" s="17" t="s">
+      <c r="B89" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="C89" s="18">
-        <v>68.349999999999994</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A90" s="17" t="s">
+      <c r="C89" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D89" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A90" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="B90" s="17" t="s">
+      <c r="B90" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="C90" s="18">
-        <v>68.349999999999994</v>
+      <c r="C90" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="D90" s="14">
+        <v>46174</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>191</v>
+      </c>
+      <c r="B91" t="s">
+        <v>192</v>
+      </c>
+      <c r="C91">
+        <v>15</v>
+      </c>
+      <c r="D91" s="14">
+        <v>46174</v>
+      </c>
+      <c r="E91" t="s">
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2114,68 +2497,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="14"/>
+      <c r="B1" s="16"/>
     </row>
     <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="9"/>
-      <c r="B9" s="10"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="9"/>
     </row>
     <row r="10" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
BigQuery: Estagio 1 completo, todos os modelos migrados
- stg_escrow, stg_order_items, stg_escrow_items e master_orders agora tem os
  dois dialetos via target.type (stg_customer_orders nao precisou mudar)
- Arrays JSON: jsonb_array_elements no SELECT vira unnest(json_query_array())
  no FROM como cross join
- master_orders: date(create_time) no lugar de ::date e cast explicito do fator
  de imposto para numeric, evitando divergencia de centavos por promocao a float
- custo_produtos: removida a linha de exemplo que sobrava nas colunas F-J da
  planilha e virava 5 colunas Unnamed no seed
- Validado modelo a modelo contra o Postgres. master_orders final identico nos
  dois: 88 linhas, GMV 3441.92, receita bruta 2022.51, 80 itens com custo
- dbt build --target bigquery: PASS=19, mesmos 19 no Postgres
</commit_message>
<xml_diff>
--- a/extraction/planilhas/custo_produtos.xlsx
+++ b/extraction/planilhas/custo_produtos.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brunoalencar/Documents/Casa e Patas/data-pipeline/extraction/planilhas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{778EAB7B-9770-AF48-A095-D20D7DF0E9C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC4F5B2-F847-F94C-B832-DCFD0E82BFA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="213">
   <si>
     <t>Custo de Produtos — Casa e Patas</t>
   </si>
@@ -55,12 +55,6 @@
   </si>
   <si>
     <t>observacao</t>
-  </si>
-  <si>
-    <t>Coleira M Azul (exemplo)</t>
-  </si>
-  <si>
-    <t>Fornecedor X, lote 45 — apague esta linha</t>
   </si>
   <si>
     <t>Como preencher a planilha custo_produtos</t>
@@ -1227,10 +1221,10 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C5" s="13">
         <v>33.770000000000003</v>
@@ -1238,25 +1232,17 @@
       <c r="D5" s="14">
         <v>46174</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="3">
-        <v>12.5</v>
-      </c>
-      <c r="I5" s="4">
-        <v>46174</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="4"/>
+      <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C6" s="13">
         <v>46.3</v>
@@ -1268,10 +1254,10 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="12" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C7" s="13">
         <v>52.57</v>
@@ -1283,10 +1269,10 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C8" s="13">
         <v>65.099999999999994</v>
@@ -1298,10 +1284,10 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C9" s="13">
         <v>33.950000000000003</v>
@@ -1313,10 +1299,10 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C10" s="13">
         <v>46.55</v>
@@ -1328,10 +1314,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C11" s="13">
         <v>52.86</v>
@@ -1343,10 +1329,10 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C12" s="13">
         <v>65.459999999999994</v>
@@ -1358,10 +1344,10 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C13" s="13">
         <v>33.950000000000003</v>
@@ -1373,10 +1359,10 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="12" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C14" s="13">
         <v>46.55</v>
@@ -1388,10 +1374,10 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C15" s="13">
         <v>52.86</v>
@@ -1403,10 +1389,10 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="12" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C16" s="13">
         <v>65.459999999999994</v>
@@ -1418,10 +1404,10 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C17" s="13">
         <v>33.950000000000003</v>
@@ -1433,10 +1419,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C18" s="13">
         <v>46.55</v>
@@ -1448,10 +1434,10 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C19" s="13">
         <v>52.86</v>
@@ -1463,10 +1449,10 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C20" s="13">
         <v>65.459999999999994</v>
@@ -1478,10 +1464,10 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C21" s="13">
         <v>33.950000000000003</v>
@@ -1493,10 +1479,10 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C22" s="13">
         <v>46.55</v>
@@ -1508,10 +1494,10 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C23" s="13">
         <v>52.86</v>
@@ -1523,10 +1509,10 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C24" s="13">
         <v>65.459999999999994</v>
@@ -1538,10 +1524,10 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="12" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C25" s="13">
         <v>33.950000000000003</v>
@@ -1553,13 +1539,13 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D26" s="14">
         <v>46174</v>
@@ -1567,13 +1553,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" s="12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D27" s="14">
         <v>46174</v>
@@ -1581,13 +1567,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A28" s="12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D28" s="14">
         <v>46174</v>
@@ -1595,13 +1581,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A29" s="12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D29" s="14">
         <v>46174</v>
@@ -1609,13 +1595,13 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D30" s="14">
         <v>46174</v>
@@ -1623,13 +1609,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C31" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D31" s="14">
         <v>46174</v>
@@ -1637,13 +1623,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C32" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D32" s="14">
         <v>46174</v>
@@ -1651,13 +1637,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A33" s="12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C33" s="13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D33" s="14">
         <v>46174</v>
@@ -1665,13 +1651,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D34" s="14">
         <v>46174</v>
@@ -1679,13 +1665,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="12" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C35" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D35" s="14">
         <v>46174</v>
@@ -1693,13 +1679,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D36" s="14">
         <v>46174</v>
@@ -1707,13 +1693,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="12" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C37" s="13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D37" s="14">
         <v>46174</v>
@@ -1721,13 +1707,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C38" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D38" s="14">
         <v>46174</v>
@@ -1735,13 +1721,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C39" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D39" s="14">
         <v>46174</v>
@@ -1749,13 +1735,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C40" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D40" s="14">
         <v>46174</v>
@@ -1763,13 +1749,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C41" s="13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D41" s="14">
         <v>46174</v>
@@ -1777,13 +1763,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D42" s="14">
         <v>46174</v>
@@ -1791,13 +1777,13 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D43" s="14">
         <v>46174</v>
@@ -1805,13 +1791,13 @@
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D44" s="14">
         <v>46174</v>
@@ -1819,13 +1805,13 @@
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="12" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D45" s="14">
         <v>46174</v>
@@ -1833,13 +1819,13 @@
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B46" s="12" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D46" s="14">
         <v>46174</v>
@@ -1847,13 +1833,13 @@
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B47" s="12" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D47" s="14">
         <v>46174</v>
@@ -1861,13 +1847,13 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B48" s="12" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D48" s="14">
         <v>46174</v>
@@ -1875,13 +1861,13 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="12" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B49" s="12" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C49" s="13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D49" s="14">
         <v>46174</v>
@@ -1889,13 +1875,13 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B50" s="12" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D50" s="14">
         <v>46174</v>
@@ -1903,13 +1889,13 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B51" s="12" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D51" s="14">
         <v>46174</v>
@@ -1917,13 +1903,13 @@
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="12" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B52" s="12" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D52" s="14">
         <v>46174</v>
@@ -1931,13 +1917,13 @@
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B53" s="12" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D53" s="14">
         <v>46174</v>
@@ -1945,13 +1931,13 @@
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D54" s="14">
         <v>46174</v>
@@ -1959,13 +1945,13 @@
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D55" s="14">
         <v>46174</v>
@@ -1973,13 +1959,13 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D56" s="14">
         <v>46174</v>
@@ -1987,13 +1973,13 @@
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B57" s="12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D57" s="14">
         <v>46174</v>
@@ -2001,13 +1987,13 @@
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D58" s="14">
         <v>46174</v>
@@ -2015,13 +2001,13 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D59" s="14">
         <v>46174</v>
@@ -2029,13 +2015,13 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D60" s="14">
         <v>46174</v>
@@ -2043,13 +2029,13 @@
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D61" s="14">
         <v>46174</v>
@@ -2057,13 +2043,13 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D62" s="14">
         <v>46174</v>
@@ -2071,13 +2057,13 @@
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A63" s="12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D63" s="14">
         <v>46174</v>
@@ -2085,13 +2071,13 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A64" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D64" s="14">
         <v>46174</v>
@@ -2099,13 +2085,13 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A65" s="12" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D65" s="14">
         <v>46174</v>
@@ -2113,13 +2099,13 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A66" s="12" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D66" s="14">
         <v>46174</v>
@@ -2127,13 +2113,13 @@
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A67" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D67" s="14">
         <v>46174</v>
@@ -2141,13 +2127,13 @@
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A68" s="12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D68" s="14">
         <v>46174</v>
@@ -2155,13 +2141,13 @@
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A69" s="12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D69" s="14">
         <v>46174</v>
@@ -2169,13 +2155,13 @@
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A70" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D70" s="14">
         <v>46174</v>
@@ -2183,13 +2169,13 @@
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A71" s="12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D71" s="14">
         <v>46174</v>
@@ -2197,13 +2183,13 @@
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A72" s="12" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D72" s="14">
         <v>46174</v>
@@ -2211,13 +2197,13 @@
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A73" s="12" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D73" s="14">
         <v>46174</v>
@@ -2225,13 +2211,13 @@
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A74" s="12" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B74" s="12" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D74" s="14">
         <v>46174</v>
@@ -2239,13 +2225,13 @@
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A75" s="12" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B75" s="12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D75" s="14">
         <v>46174</v>
@@ -2253,13 +2239,13 @@
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A76" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B76" s="12" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D76" s="14">
         <v>46174</v>
@@ -2267,13 +2253,13 @@
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A77" s="12" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B77" s="12" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D77" s="14">
         <v>46174</v>
@@ -2281,13 +2267,13 @@
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A78" s="12" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B78" s="12" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D78" s="14">
         <v>46174</v>
@@ -2295,13 +2281,13 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A79" s="12" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B79" s="12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D79" s="14">
         <v>46174</v>
@@ -2309,13 +2295,13 @@
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A80" s="12" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B80" s="12" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D80" s="14">
         <v>46174</v>
@@ -2323,13 +2309,13 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A81" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B81" s="12" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D81" s="14">
         <v>46174</v>
@@ -2337,13 +2323,13 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A82" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B82" s="12" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D82" s="14">
         <v>46174</v>
@@ -2351,13 +2337,13 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A83" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B83" s="12" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D83" s="14">
         <v>46174</v>
@@ -2365,13 +2351,13 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A84" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B84" s="12" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D84" s="14">
         <v>46174</v>
@@ -2379,13 +2365,13 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A85" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B85" s="12" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D85" s="14">
         <v>46174</v>
@@ -2393,13 +2379,13 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A86" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B86" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D86" s="14">
         <v>46174</v>
@@ -2407,13 +2393,13 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B87" s="12" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C87" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D87" s="14">
         <v>46174</v>
@@ -2421,13 +2407,13 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" s="12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B88" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D88" s="14">
         <v>46174</v>
@@ -2435,13 +2421,13 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B89" s="12" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D89" s="14">
         <v>46174</v>
@@ -2449,13 +2435,13 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B90" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C90" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D90" s="14">
         <v>46174</v>
@@ -2463,10 +2449,10 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B91" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C91">
         <v>15</v>
@@ -2475,7 +2461,7 @@
         <v>46174</v>
       </c>
       <c r="E91" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2498,16 +2484,16 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="18" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B1" s="16"/>
     </row>
     <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2515,7 +2501,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2523,7 +2509,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2531,7 +2517,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2539,7 +2525,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2547,7 +2533,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -2556,10 +2542,10 @@
     </row>
     <row r="10" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>